<commit_message>
Add factory selection, optimize PDF generation, and enhance email features
</commit_message>
<xml_diff>
--- a/鑄件盤點資料.xlsx
+++ b/鑄件盤點資料.xlsx
@@ -8654,13 +8654,13 @@
         <v>0</v>
       </c>
       <c r="D2" s="47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="47" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" s="47" t="inlineStr"/>
       <c r="H2" s="47" t="n">
@@ -9019,7 +9019,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G13" s="47" t="inlineStr"/>
       <c r="H13" s="47" t="n">
@@ -9329,7 +9329,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" s="47" t="n">
         <v>0</v>
@@ -9362,20 +9362,20 @@
         </is>
       </c>
       <c r="C23" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="47" t="n">
-        <v>0</v>
-      </c>
       <c r="F23" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="47" t="inlineStr"/>
       <c r="H23" s="47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23" s="47" t="inlineStr"/>
       <c r="J23" s="47" t="inlineStr"/>
@@ -9438,20 +9438,20 @@
         </is>
       </c>
       <c r="C25" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="47" t="n">
         <v>1</v>
-      </c>
-      <c r="D25" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="47" t="n">
-        <v>0</v>
       </c>
       <c r="F25" s="47" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="47" t="inlineStr"/>
       <c r="H25" s="47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" s="47" t="inlineStr"/>
       <c r="J25" s="47" t="inlineStr"/>
@@ -9628,13 +9628,13 @@
         <v>0</v>
       </c>
       <c r="D30" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="47" t="n">
         <v>1</v>
-      </c>
-      <c r="E30" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="47" t="n">
-        <v>0</v>
       </c>
       <c r="G30" s="47" t="inlineStr"/>
       <c r="H30" s="47" t="n">
@@ -9700,7 +9700,7 @@
         <v>0</v>
       </c>
       <c r="D32" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E32" s="47" t="n">
         <v>0</v>
@@ -9733,7 +9733,7 @@
         <v>0</v>
       </c>
       <c r="D33" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" s="47" t="n">
         <v>0</v>
@@ -10211,13 +10211,13 @@
         </is>
       </c>
       <c r="C48" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="47" t="n">
         <v>1</v>
-      </c>
-      <c r="D48" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="47" t="n">
-        <v>0</v>
       </c>
       <c r="F48" s="47" t="n">
         <v>0</v>
@@ -10246,10 +10246,10 @@
         </is>
       </c>
       <c r="C49" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="47" t="n">
         <v>1</v>
-      </c>
-      <c r="D49" s="47" t="n">
-        <v>0</v>
       </c>
       <c r="E49" s="47" t="n">
         <v>0</v>
@@ -10312,7 +10312,7 @@
         </is>
       </c>
       <c r="C51" s="47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" s="47" t="n">
         <v>0</v>
@@ -10321,7 +10321,7 @@
         <v>0</v>
       </c>
       <c r="F51" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G51" s="47" t="inlineStr"/>
       <c r="H51" s="47" t="n">
@@ -10353,10 +10353,10 @@
         <v>0</v>
       </c>
       <c r="E52" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="47" t="n">
         <v>1</v>
-      </c>
-      <c r="F52" s="47" t="n">
-        <v>0</v>
       </c>
       <c r="G52" s="47" t="inlineStr"/>
       <c r="H52" s="47" t="n">
@@ -10737,7 +10737,7 @@
     </row>
     <row r="64">
       <c r="A64" s="47" t="n">
-        <v>8810000964</v>
+        <v>8810000957</v>
       </c>
       <c r="B64" s="47" t="inlineStr">
         <is>
@@ -10745,20 +10745,20 @@
         </is>
       </c>
       <c r="C64" s="47" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D64" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E64" s="47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F64" s="47" t="n">
         <v>0</v>
       </c>
       <c r="G64" s="47" t="inlineStr"/>
       <c r="H64" s="47" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I64" s="47" t="inlineStr"/>
       <c r="J64" s="47" t="inlineStr"/>
@@ -10809,13 +10809,13 @@
         </is>
       </c>
       <c r="C66" s="47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D66" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E66" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F66" s="47" t="n">
         <v>0</v>
@@ -11373,7 +11373,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H6" s="47" t="n">
         <v>1</v>
@@ -11449,12 +11449,18 @@
       <c r="E8" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="47" t="inlineStr"/>
-      <c r="G8" s="47" t="inlineStr"/>
+      <c r="F8" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="47" t="n">
+        <v>1</v>
+      </c>
       <c r="H8" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="47" t="inlineStr"/>
+      <c r="I8" s="47" t="n">
+        <v>1</v>
+      </c>
       <c r="J8" s="47" t="inlineStr"/>
       <c r="K8" s="47" t="inlineStr"/>
       <c r="L8" s="47" t="n">
@@ -11613,7 +11619,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" s="47" t="n">
         <v>0</v>
@@ -11676,7 +11682,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E14" s="47" t="n">
         <v>0</v>
@@ -11962,12 +11968,18 @@
       <c r="E21" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="47" t="inlineStr"/>
-      <c r="G21" s="47" t="inlineStr"/>
+      <c r="F21" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="47" t="n">
+        <v>0</v>
+      </c>
       <c r="H21" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="47" t="inlineStr"/>
+      <c r="I21" s="47" t="n">
+        <v>1</v>
+      </c>
       <c r="J21" s="47" t="inlineStr"/>
       <c r="K21" s="47" t="inlineStr"/>
       <c r="L21" s="47" t="inlineStr"/>
@@ -12121,7 +12133,7 @@
         </is>
       </c>
       <c r="C26" s="47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="47" t="n">
         <v>0</v>
@@ -12133,7 +12145,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H26" s="47" t="n">
         <v>1</v>
@@ -12244,18 +12256,20 @@
         <v>0</v>
       </c>
       <c r="E29" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="47" t="n">
-        <v>0</v>
-      </c>
       <c r="H29" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="I29" s="47" t="inlineStr"/>
+      <c r="I29" s="47" t="n">
+        <v>3</v>
+      </c>
       <c r="J29" s="47" t="n">
         <v>3</v>
       </c>
@@ -12639,7 +12653,7 @@
         <v>0</v>
       </c>
       <c r="D39" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E39" s="47" t="n">
         <v>0</v>
@@ -12653,7 +12667,9 @@
       <c r="H39" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="I39" s="47" t="inlineStr"/>
+      <c r="I39" s="47" t="n">
+        <v>0</v>
+      </c>
       <c r="J39" s="47" t="n">
         <v>1</v>
       </c>
@@ -12796,7 +12812,7 @@
         </is>
       </c>
       <c r="C43" s="47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D43" s="47" t="n">
         <v>0</v>
@@ -12808,7 +12824,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H43" s="47" t="n">
         <v>0</v>
@@ -13064,13 +13080,13 @@
       </c>
       <c r="D4" s="47" t="inlineStr"/>
       <c r="E4" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="47" t="n">
         <v>1</v>
-      </c>
-      <c r="F4" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="47" t="n">
-        <v>0</v>
       </c>
       <c r="H4" s="47" t="inlineStr"/>
       <c r="I4" s="47" t="n">
@@ -13184,7 +13200,7 @@
         </is>
       </c>
       <c r="C8" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="47" t="inlineStr"/>
       <c r="E8" s="47" t="n">
@@ -13197,7 +13213,9 @@
         <v>0</v>
       </c>
       <c r="H8" s="47" t="inlineStr"/>
-      <c r="I8" s="47" t="inlineStr"/>
+      <c r="I8" s="47" t="n">
+        <v>1</v>
+      </c>
       <c r="J8" s="47" t="inlineStr"/>
       <c r="K8" s="47" t="inlineStr"/>
       <c r="L8" s="47" t="inlineStr">
@@ -13284,7 +13302,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H10" s="47" t="inlineStr"/>
       <c r="I10" s="47" t="n">
@@ -13428,11 +13446,11 @@
         <v>0</v>
       </c>
       <c r="G13" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="47" t="inlineStr"/>
       <c r="I13" s="47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13" s="47" t="inlineStr"/>
       <c r="K13" s="47" t="n">
@@ -13481,7 +13499,9 @@
         <v>2</v>
       </c>
       <c r="H14" s="47" t="inlineStr"/>
-      <c r="I14" s="47" t="inlineStr"/>
+      <c r="I14" s="47" t="n">
+        <v>2</v>
+      </c>
       <c r="J14" s="47" t="inlineStr"/>
       <c r="K14" s="47" t="inlineStr"/>
       <c r="L14" s="47" t="inlineStr">
@@ -13816,458 +13836,466 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="47" t="inlineStr"/>
+      <c r="B2" s="47" t="inlineStr">
         <is>
           <t>5BC-4300</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="n">
+      <c r="D2" s="47" t="inlineStr"/>
+      <c r="E2" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="F2" s="47" t="inlineStr"/>
+      <c r="G2" s="47" t="inlineStr"/>
+      <c r="H2" s="47" t="inlineStr"/>
+      <c r="I2" s="47" t="inlineStr"/>
+      <c r="J2" s="47" t="inlineStr"/>
+      <c r="K2" s="47" t="inlineStr"/>
+      <c r="L2" s="47" t="inlineStr"/>
+      <c r="M2" s="47" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr">
+      <c r="A3" s="47" t="inlineStr"/>
+      <c r="B3" s="47" t="inlineStr">
         <is>
           <t>HEP2150-1720</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="n">
+      <c r="C3" s="47" t="inlineStr"/>
+      <c r="D3" s="47" t="inlineStr"/>
+      <c r="E3" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+      <c r="F3" s="47" t="inlineStr"/>
+      <c r="G3" s="47" t="inlineStr"/>
+      <c r="H3" s="47" t="inlineStr"/>
+      <c r="I3" s="47" t="inlineStr"/>
+      <c r="J3" s="47" t="inlineStr"/>
+      <c r="K3" s="47" t="inlineStr"/>
+      <c r="L3" s="47" t="inlineStr"/>
+      <c r="M3" s="47" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr"/>
+      <c r="B4" s="47" t="inlineStr">
         <is>
           <t>HEP2150-1620</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="E4" s="47" t="inlineStr"/>
+      <c r="F4" s="47" t="inlineStr"/>
+      <c r="G4" s="47" t="inlineStr"/>
+      <c r="H4" s="47" t="inlineStr"/>
+      <c r="I4" s="47" t="inlineStr"/>
+      <c r="J4" s="47" t="inlineStr"/>
+      <c r="K4" s="47" t="inlineStr"/>
+      <c r="L4" s="47" t="inlineStr"/>
+      <c r="M4" s="47" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr"/>
+      <c r="B5" s="47" t="inlineStr">
         <is>
           <t>HSA4265</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="D5" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="47" t="inlineStr"/>
+      <c r="G5" s="47" t="inlineStr"/>
+      <c r="H5" s="47" t="inlineStr"/>
+      <c r="I5" s="47" t="inlineStr"/>
+      <c r="J5" s="47" t="inlineStr"/>
+      <c r="K5" s="47" t="inlineStr"/>
+      <c r="L5" s="47" t="inlineStr"/>
+      <c r="M5" s="47" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>8811001091</v>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
+        <is>
+          <t>8811001113</t>
+        </is>
+      </c>
+      <c r="B6" s="47" t="inlineStr">
         <is>
           <t>LG-800</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>8</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="C6" s="47" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="47" t="n">
+        <v>9</v>
+      </c>
+      <c r="H6" s="47" t="inlineStr"/>
+      <c r="I6" s="47" t="inlineStr"/>
+      <c r="J6" s="47" t="inlineStr"/>
+      <c r="K6" s="47" t="inlineStr"/>
+      <c r="L6" s="47" t="inlineStr"/>
+      <c r="M6" s="47" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="47" t="n">
         <v>8811001273</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="47" t="inlineStr">
         <is>
           <t>LG-1370</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="C7" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="47" t="inlineStr"/>
+      <c r="H7" s="47" t="inlineStr"/>
+      <c r="I7" s="47" t="inlineStr"/>
+      <c r="J7" s="47" t="inlineStr"/>
+      <c r="K7" s="47" t="inlineStr"/>
+      <c r="L7" s="47" t="inlineStr"/>
+      <c r="M7" s="47" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="47" t="n">
         <v>8811001013</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>MVP-860</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="C8" s="47" t="inlineStr"/>
+      <c r="D8" s="47" t="inlineStr"/>
+      <c r="E8" s="47" t="inlineStr"/>
+      <c r="F8" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="47" t="inlineStr"/>
+      <c r="H8" s="47" t="inlineStr"/>
+      <c r="I8" s="47" t="inlineStr"/>
+      <c r="J8" s="47" t="inlineStr"/>
+      <c r="K8" s="47" t="inlineStr"/>
+      <c r="L8" s="47" t="inlineStr"/>
+      <c r="M8" s="47" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="47" t="n">
         <v>8811001077</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="47" t="inlineStr">
         <is>
           <t>MVP-860+200H</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="47" t="inlineStr"/>
+      <c r="I9" s="47" t="inlineStr"/>
+      <c r="J9" s="47" t="inlineStr"/>
+      <c r="K9" s="47" t="inlineStr"/>
+      <c r="L9" s="47" t="inlineStr"/>
+      <c r="M9" s="47" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="47" t="n">
+        <v>8811001393</v>
+      </c>
+      <c r="B10" s="47" t="inlineStr">
+        <is>
+          <t>MVP-11</t>
+        </is>
+      </c>
+      <c r="C10" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="47" t="inlineStr"/>
+      <c r="I10" s="47" t="inlineStr"/>
+      <c r="J10" s="47" t="inlineStr"/>
+      <c r="K10" s="47" t="inlineStr"/>
+      <c r="L10" s="47" t="inlineStr"/>
+      <c r="M10" s="47" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="47" t="n">
+        <v>8811001536</v>
+      </c>
+      <c r="B11" s="47" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="C11" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="47" t="inlineStr"/>
+      <c r="H11" s="47" t="inlineStr"/>
+      <c r="I11" s="47" t="inlineStr"/>
+      <c r="J11" s="47" t="inlineStr"/>
+      <c r="K11" s="47" t="inlineStr"/>
+      <c r="L11" s="47" t="inlineStr"/>
+      <c r="M11" s="47" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="47" t="n">
+        <v>8811001338</v>
+      </c>
+      <c r="B12" s="47" t="inlineStr">
+        <is>
+          <t>S-PLUS 8</t>
+        </is>
+      </c>
+      <c r="C12" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="47" t="inlineStr"/>
+      <c r="F12" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="47" t="inlineStr"/>
+      <c r="H12" s="47" t="inlineStr"/>
+      <c r="I12" s="47" t="inlineStr"/>
+      <c r="J12" s="47" t="inlineStr"/>
+      <c r="K12" s="47" t="inlineStr"/>
+      <c r="L12" s="47" t="inlineStr"/>
+      <c r="M12" s="47" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="47" t="n">
+        <v>8811001526</v>
+      </c>
+      <c r="B13" s="47" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="C13" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="47" t="inlineStr"/>
+      <c r="I13" s="47" t="inlineStr"/>
+      <c r="J13" s="47" t="inlineStr"/>
+      <c r="K13" s="47" t="inlineStr"/>
+      <c r="L13" s="47" t="inlineStr"/>
+      <c r="M13" s="47" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="47" t="n">
+        <v>8811001616</v>
+      </c>
+      <c r="B14" s="47" t="inlineStr">
+        <is>
+          <t>LG-1370-NEO</t>
+        </is>
+      </c>
+      <c r="C14" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>8811001393</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>MVP-11</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>8811001536</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>A10</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>8811001338</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>S-PLUS 8</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>8811001526</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>S8</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
+      <c r="D14" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="47" t="inlineStr"/>
+      <c r="J14" s="47" t="inlineStr"/>
+      <c r="K14" s="47" t="inlineStr">
+        <is>
+          <t>M1:14.5HR</t>
+        </is>
+      </c>
+      <c r="L14" s="47" t="inlineStr">
+        <is>
+          <t>M2:7.5HR</t>
+        </is>
+      </c>
+      <c r="M14" s="47" t="inlineStr">
+        <is>
+          <t>M7:2.HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="47" t="n">
+        <v>8811001625</v>
+      </c>
+      <c r="B15" s="47" t="inlineStr">
+        <is>
+          <t>LG-1370-NEO+200H</t>
+        </is>
+      </c>
+      <c r="C15" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="47" t="inlineStr"/>
+      <c r="J15" s="47" t="inlineStr"/>
+      <c r="K15" s="47" t="inlineStr"/>
+      <c r="L15" s="47" t="inlineStr"/>
+      <c r="M15" s="47" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="47" t="n">
+        <v>8811001619</v>
+      </c>
+      <c r="B16" s="47" t="inlineStr">
+        <is>
+          <t>LG-1000-NEO</t>
+        </is>
+      </c>
+      <c r="C16" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
+      <c r="D16" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="47" t="inlineStr"/>
+      <c r="H16" s="47" t="inlineStr"/>
+      <c r="I16" s="47" t="inlineStr"/>
+      <c r="J16" s="47" t="inlineStr"/>
+      <c r="K16" s="47" t="inlineStr"/>
+      <c r="L16" s="47" t="inlineStr"/>
+      <c r="M16" s="47" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="47" t="n">
+        <v>8811001623</v>
+      </c>
+      <c r="B17" s="47" t="inlineStr">
+        <is>
+          <t>LG-1000-NEO+200H</t>
+        </is>
+      </c>
+      <c r="C17" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>8811001616</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>LG-1370-NEO</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>M1:14.5HR</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>M2:7.5HR</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>M7:2.HR</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>8811001625</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>LG-1370-NEO+200H</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>8811001619</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>LG-1000-NEO</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>8811001623</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>LG-1000-NEO+200H</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+      <c r="D17" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="47" t="inlineStr"/>
+      <c r="H17" s="47" t="inlineStr"/>
+      <c r="I17" s="47" t="inlineStr"/>
+      <c r="J17" s="47" t="inlineStr"/>
+      <c r="K17" s="47" t="inlineStr"/>
+      <c r="L17" s="47" t="inlineStr"/>
+      <c r="M17" s="47" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>